<commit_message>
chore: update Template_ABRASCRM.xlsx with latest formatting updates
</commit_message>
<xml_diff>
--- a/app/templates/informes/Informes agregado/Abrass/Template_ABRASCRM.xlsx
+++ b/app/templates/informes/Informes agregado/Abrass/Template_ABRASCRM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\3.0 Formatos e informes\2026\1.0 Informe de ensayo\1.2 Informe agregados\INFORME ACREDITADO-E ISO\1.1 JUNIO 15-06-26\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\informes\Informes agregado\Abrass\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2582D75-BDDD-458A-B201-47BECC238717}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85F5FB35-E5C0-427C-9E95-D228F30D744B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO" sheetId="96" r:id="rId1"/>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="209">
   <si>
     <t>:</t>
   </si>
@@ -892,6 +892,12 @@
   </si>
   <si>
     <t>TIPO DE MUESTRA**</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>NO</t>
   </si>
 </sst>
 </file>
@@ -2996,12 +3002,6 @@
     <xf numFmtId="17" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="11" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
       <protection hidden="1"/>
@@ -3133,18 +3133,162 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="19" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="2" borderId="9" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="2" borderId="8" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="9" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="8" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="9" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="8" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="9" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="14" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="8" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="12" fontId="20" fillId="2" borderId="9" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="12" fontId="20" fillId="2" borderId="8" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="12" fontId="13" fillId="2" borderId="9" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="12" fontId="13" fillId="2" borderId="8" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="9" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="8" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="2" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="9" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="8" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="14" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
@@ -3164,150 +3308,37 @@
       <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="9" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="8" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="9" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="8" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="14" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="9" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="8" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="20" fillId="2" borderId="9" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="20" fillId="2" borderId="8" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="20" fillId="2" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="12" fontId="13" fillId="2" borderId="9" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="12" fontId="13" fillId="2" borderId="8" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="9" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="8" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="9" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="14" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="8" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="12" fontId="20" fillId="2" borderId="9" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="12" fontId="20" fillId="2" borderId="8" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="19" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="6" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="6" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3328,33 +3359,54 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="17" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="17" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="6" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -3369,79 +3421,6 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="17" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="17" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="40" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="40" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="3" fillId="2" borderId="9" xfId="4" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="3" fillId="2" borderId="8" xfId="4" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="44" fillId="2" borderId="4" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3502,6 +3481,30 @@
     <xf numFmtId="0" fontId="51" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="40" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="40" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="3" fillId="2" borderId="9" xfId="4" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="3" fillId="2" borderId="8" xfId="4" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="41" fillId="2" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3525,6 +3528,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -3788,7 +3794,7 @@
                 <a:cs typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="es-ES"/>
+            <a:endParaRPr lang="es-PE"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="145561856"/>
@@ -3825,7 +3831,7 @@
                 <a:cs typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="es-ES"/>
+            <a:endParaRPr lang="es-PE"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="145560320"/>
@@ -3863,7 +3869,7 @@
           <a:cs typeface="Calibri"/>
         </a:defRPr>
       </a:pPr>
-      <a:endParaRPr lang="es-ES"/>
+      <a:endParaRPr lang="es-PE"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -4142,144 +4148,6 @@
         </a:ln>
       </xdr:spPr>
     </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>457200</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>295275</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="14" name="CuadroTexto 13">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4C37FF8C-B306-4DFF-88BF-20BAB7B4365D}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6349365" y="2941320"/>
-          <a:ext cx="447675" cy="295275"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:solidFill>
-            <a:sysClr val="windowText" lastClr="000000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="es-PE" sz="1100"/>
-            <a:t>SI</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>466725</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>219075</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="15" name="CuadroTexto 14">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{838F02D4-179E-4E31-8641-3EF1E9EAC97B}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6806565" y="2950845"/>
-          <a:ext cx="445770" cy="295275"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:solidFill>
-            <a:sysClr val="windowText" lastClr="000000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="es-PE" sz="1100"/>
-            <a:t>NO</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
@@ -5810,7 +5678,7 @@
     <col min="8" max="8" width="10.109375" style="406" customWidth="1"/>
     <col min="9" max="9" width="11.109375" style="406" customWidth="1"/>
     <col min="10" max="10" width="10.109375" style="406" customWidth="1"/>
-    <col min="11" max="11" width="3.44140625" style="406" customWidth="1"/>
+    <col min="11" max="11" width="9.109375" style="406" customWidth="1"/>
     <col min="12" max="12" width="6.44140625" style="406" customWidth="1"/>
     <col min="13" max="13" width="18.77734375" style="406" customWidth="1"/>
     <col min="14" max="14" width="20.5546875" style="406" customWidth="1"/>
@@ -5848,10 +5716,10 @@
       <c r="I2" s="386"/>
       <c r="J2" s="386"/>
       <c r="K2" s="408"/>
-      <c r="M2" s="456" t="s">
+      <c r="M2" s="454" t="s">
         <v>201</v>
       </c>
-      <c r="N2" s="457"/>
+      <c r="N2" s="455"/>
     </row>
     <row r="3" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="407"/>
@@ -5865,10 +5733,10 @@
       <c r="I3" s="386"/>
       <c r="J3" s="386"/>
       <c r="K3" s="408"/>
-      <c r="M3" s="456" t="s">
+      <c r="M3" s="454" t="s">
         <v>202</v>
       </c>
-      <c r="N3" s="458"/>
+      <c r="N3" s="456"/>
     </row>
     <row r="4" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="407"/>
@@ -5882,10 +5750,10 @@
       <c r="I4" s="386"/>
       <c r="J4" s="386"/>
       <c r="K4" s="408"/>
-      <c r="M4" s="456" t="s">
+      <c r="M4" s="454" t="s">
         <v>203</v>
       </c>
-      <c r="N4" s="458"/>
+      <c r="N4" s="456"/>
     </row>
     <row r="5" spans="1:24" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="409"/>
@@ -5899,10 +5767,10 @@
       <c r="I5" s="410"/>
       <c r="J5" s="410"/>
       <c r="K5" s="411"/>
-      <c r="M5" s="456" t="s">
+      <c r="M5" s="454" t="s">
         <v>44</v>
       </c>
-      <c r="N5" s="458"/>
+      <c r="N5" s="456"/>
     </row>
     <row r="6" spans="1:24" ht="7.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B6" s="412"/>
@@ -5915,51 +5783,51 @@
       <c r="I6" s="412"/>
       <c r="J6" s="412"/>
       <c r="K6" s="412"/>
-      <c r="M6" s="459"/>
-      <c r="N6" s="460"/>
+      <c r="M6" s="457"/>
+      <c r="N6" s="458"/>
     </row>
     <row r="7" spans="1:24" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="511" t="s">
+      <c r="A7" s="464" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="511"/>
-      <c r="C7" s="511"/>
-      <c r="D7" s="511"/>
-      <c r="E7" s="511"/>
-      <c r="F7" s="511"/>
-      <c r="G7" s="511"/>
-      <c r="H7" s="511"/>
-      <c r="I7" s="511"/>
-      <c r="J7" s="511"/>
-      <c r="K7" s="511"/>
-      <c r="M7" s="456" t="s">
+      <c r="B7" s="464"/>
+      <c r="C7" s="464"/>
+      <c r="D7" s="464"/>
+      <c r="E7" s="464"/>
+      <c r="F7" s="464"/>
+      <c r="G7" s="464"/>
+      <c r="H7" s="464"/>
+      <c r="I7" s="464"/>
+      <c r="J7" s="464"/>
+      <c r="K7" s="464"/>
+      <c r="M7" s="454" t="s">
         <v>132</v>
       </c>
-      <c r="N7" s="460"/>
+      <c r="N7" s="458"/>
     </row>
     <row r="8" spans="1:24" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="512" t="s">
+      <c r="A8" s="465" t="s">
         <v>174</v>
       </c>
-      <c r="B8" s="512"/>
-      <c r="C8" s="512"/>
-      <c r="D8" s="512"/>
-      <c r="E8" s="512"/>
-      <c r="F8" s="512"/>
-      <c r="G8" s="512"/>
-      <c r="H8" s="512"/>
-      <c r="I8" s="512"/>
-      <c r="J8" s="512"/>
-      <c r="K8" s="512"/>
-      <c r="M8" s="456" t="s">
+      <c r="B8" s="465"/>
+      <c r="C8" s="465"/>
+      <c r="D8" s="465"/>
+      <c r="E8" s="465"/>
+      <c r="F8" s="465"/>
+      <c r="G8" s="465"/>
+      <c r="H8" s="465"/>
+      <c r="I8" s="465"/>
+      <c r="J8" s="465"/>
+      <c r="K8" s="465"/>
+      <c r="M8" s="454" t="s">
         <v>21</v>
       </c>
-      <c r="N8" s="461"/>
-      <c r="S8" s="513"/>
-      <c r="T8" s="513"/>
-      <c r="U8" s="513"/>
-      <c r="V8" s="513"/>
-      <c r="W8" s="513"/>
+      <c r="N8" s="459"/>
+      <c r="S8" s="466"/>
+      <c r="T8" s="466"/>
+      <c r="U8" s="466"/>
+      <c r="V8" s="466"/>
+      <c r="W8" s="466"/>
       <c r="X8" s="413"/>
     </row>
     <row r="9" spans="1:24" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -5973,52 +5841,52 @@
       <c r="I9" s="414"/>
       <c r="J9" s="414"/>
       <c r="K9" s="414"/>
-      <c r="M9" s="456" t="s">
+      <c r="M9" s="454" t="s">
         <v>204</v>
       </c>
-      <c r="N9" s="460"/>
-      <c r="S9" s="513"/>
-      <c r="T9" s="513"/>
-      <c r="U9" s="513"/>
-      <c r="V9" s="513"/>
-      <c r="W9" s="513"/>
+      <c r="N9" s="458"/>
+      <c r="S9" s="466"/>
+      <c r="T9" s="466"/>
+      <c r="U9" s="466"/>
+      <c r="V9" s="466"/>
+      <c r="W9" s="466"/>
       <c r="X9" s="413"/>
     </row>
     <row r="10" spans="1:24" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="415"/>
-      <c r="C10" s="431" t="s">
+      <c r="C10" s="429" t="s">
         <v>197</v>
       </c>
-      <c r="D10" s="467" t="s">
+      <c r="D10" s="500" t="s">
         <v>198</v>
       </c>
-      <c r="E10" s="468"/>
-      <c r="F10" s="466" t="s">
+      <c r="E10" s="502"/>
+      <c r="F10" s="508" t="s">
         <v>199</v>
       </c>
-      <c r="G10" s="466"/>
-      <c r="H10" s="466" t="s">
+      <c r="G10" s="508"/>
+      <c r="H10" s="508" t="s">
         <v>200</v>
       </c>
-      <c r="I10" s="466"/>
+      <c r="I10" s="508"/>
       <c r="K10" s="414"/>
-      <c r="M10" s="459"/>
-      <c r="N10" s="460"/>
+      <c r="M10" s="457"/>
+      <c r="N10" s="458"/>
     </row>
     <row r="11" spans="1:24" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="415"/>
-      <c r="C11" s="431"/>
-      <c r="D11" s="467"/>
-      <c r="E11" s="468"/>
-      <c r="F11" s="466"/>
-      <c r="G11" s="466"/>
-      <c r="H11" s="466"/>
-      <c r="I11" s="466"/>
+      <c r="C11" s="429"/>
+      <c r="D11" s="500"/>
+      <c r="E11" s="502"/>
+      <c r="F11" s="508"/>
+      <c r="G11" s="508"/>
+      <c r="H11" s="508"/>
+      <c r="I11" s="508"/>
       <c r="K11" s="414"/>
-      <c r="M11" s="456" t="s">
+      <c r="M11" s="454" t="s">
         <v>49</v>
       </c>
-      <c r="N11" s="460"/>
+      <c r="N11" s="458"/>
       <c r="P11" s="417"/>
       <c r="Q11" s="418"/>
     </row>
@@ -6033,50 +5901,50 @@
       <c r="I12" s="419"/>
       <c r="J12" s="419"/>
       <c r="K12" s="414"/>
-      <c r="M12" s="456" t="s">
+      <c r="M12" s="454" t="s">
         <v>22</v>
       </c>
-      <c r="N12" s="461"/>
-      <c r="P12" s="502"/>
-      <c r="Q12" s="502"/>
+      <c r="N12" s="459"/>
+      <c r="P12" s="467"/>
+      <c r="Q12" s="467"/>
     </row>
     <row r="13" spans="1:24" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="503" t="s">
+      <c r="A13" s="468" t="s">
         <v>175</v>
       </c>
-      <c r="B13" s="504"/>
-      <c r="C13" s="504"/>
-      <c r="D13" s="504"/>
-      <c r="E13" s="504"/>
-      <c r="F13" s="504"/>
-      <c r="G13" s="504"/>
-      <c r="H13" s="504"/>
-      <c r="I13" s="504"/>
-      <c r="J13" s="504"/>
-      <c r="K13" s="505"/>
+      <c r="B13" s="469"/>
+      <c r="C13" s="469"/>
+      <c r="D13" s="469"/>
+      <c r="E13" s="469"/>
+      <c r="F13" s="469"/>
+      <c r="G13" s="469"/>
+      <c r="H13" s="469"/>
+      <c r="I13" s="469"/>
+      <c r="J13" s="469"/>
+      <c r="K13" s="470"/>
       <c r="L13" s="416"/>
-      <c r="M13" s="456" t="s">
+      <c r="M13" s="454" t="s">
         <v>23</v>
       </c>
-      <c r="N13" s="461"/>
+      <c r="N13" s="459"/>
     </row>
     <row r="14" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="506" t="s">
+      <c r="A14" s="471" t="s">
         <v>176</v>
       </c>
-      <c r="B14" s="507"/>
-      <c r="C14" s="507"/>
-      <c r="D14" s="507"/>
-      <c r="E14" s="507"/>
-      <c r="F14" s="507"/>
-      <c r="G14" s="507"/>
-      <c r="H14" s="507"/>
-      <c r="I14" s="507"/>
-      <c r="J14" s="507"/>
-      <c r="K14" s="508"/>
+      <c r="B14" s="472"/>
+      <c r="C14" s="472"/>
+      <c r="D14" s="472"/>
+      <c r="E14" s="472"/>
+      <c r="F14" s="472"/>
+      <c r="G14" s="472"/>
+      <c r="H14" s="472"/>
+      <c r="I14" s="472"/>
+      <c r="J14" s="472"/>
+      <c r="K14" s="473"/>
       <c r="L14" s="416"/>
-      <c r="M14" s="459"/>
-      <c r="N14" s="460"/>
+      <c r="M14" s="457"/>
+      <c r="N14" s="458"/>
     </row>
     <row r="15" spans="1:24" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="415"/>
@@ -6090,10 +5958,10 @@
       <c r="J15" s="420"/>
       <c r="K15" s="421"/>
       <c r="L15" s="416"/>
-      <c r="M15" s="456" t="s">
+      <c r="M15" s="454" t="s">
         <v>45</v>
       </c>
-      <c r="N15" s="462"/>
+      <c r="N15" s="460"/>
     </row>
     <row r="16" spans="1:24" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="415"/>
@@ -6107,53 +5975,57 @@
       <c r="J16" s="420"/>
       <c r="K16" s="421"/>
       <c r="L16" s="416"/>
-      <c r="M16" s="456" t="s">
+      <c r="M16" s="454" t="s">
         <v>205</v>
       </c>
-      <c r="N16" s="462"/>
+      <c r="N16" s="460"/>
     </row>
     <row r="17" spans="2:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="481" t="s">
+      <c r="B17" s="474" t="s">
         <v>51</v>
       </c>
-      <c r="C17" s="482"/>
+      <c r="C17" s="475"/>
       <c r="D17" s="284" t="s">
         <v>38</v>
       </c>
-      <c r="E17" s="483" t="s">
+      <c r="E17" s="476" t="s">
         <v>37</v>
       </c>
-      <c r="F17" s="484"/>
+      <c r="F17" s="477"/>
       <c r="G17" s="387"/>
-      <c r="H17" s="509" t="s">
+      <c r="H17" s="478" t="s">
         <v>177</v>
       </c>
-      <c r="I17" s="510"/>
-      <c r="J17" s="422"/>
-      <c r="K17" s="423"/>
+      <c r="I17" s="479"/>
+      <c r="J17" s="463" t="s">
+        <v>207</v>
+      </c>
+      <c r="K17" s="584" t="s">
+        <v>208</v>
+      </c>
       <c r="L17" s="416"/>
-      <c r="M17" s="456" t="s">
+      <c r="M17" s="454" t="s">
         <v>206</v>
       </c>
-      <c r="N17" s="463"/>
+      <c r="N17" s="461"/>
     </row>
     <row r="18" spans="2:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="478" t="s">
+      <c r="B18" s="480" t="s">
         <v>52</v>
       </c>
-      <c r="C18" s="479"/>
+      <c r="C18" s="481"/>
       <c r="D18" s="61" t="s">
         <v>39</v>
       </c>
-      <c r="E18" s="475"/>
-      <c r="F18" s="476"/>
+      <c r="E18" s="482"/>
+      <c r="F18" s="483"/>
       <c r="G18" s="388"/>
-      <c r="H18" s="499" t="s">
+      <c r="H18" s="484" t="s">
         <v>131</v>
       </c>
-      <c r="I18" s="499"/>
-      <c r="J18" s="500"/>
-      <c r="K18" s="500"/>
+      <c r="I18" s="484"/>
+      <c r="J18" s="485"/>
+      <c r="K18" s="485"/>
       <c r="L18" s="416"/>
       <c r="M18" s="416"/>
     </row>
@@ -6165,14 +6037,14 @@
       <c r="D19" s="391" t="s">
         <v>39</v>
       </c>
-      <c r="E19" s="475"/>
-      <c r="F19" s="476"/>
-      <c r="H19" s="501" t="s">
+      <c r="E19" s="482"/>
+      <c r="F19" s="483"/>
+      <c r="H19" s="486" t="s">
         <v>178</v>
       </c>
-      <c r="I19" s="501"/>
-      <c r="J19" s="501"/>
-      <c r="K19" s="501"/>
+      <c r="I19" s="486"/>
+      <c r="J19" s="486"/>
+      <c r="K19" s="486"/>
       <c r="L19" s="416"/>
       <c r="M19" s="416"/>
     </row>
@@ -6184,8 +6056,8 @@
       <c r="D20" s="61" t="s">
         <v>39</v>
       </c>
-      <c r="E20" s="475"/>
-      <c r="F20" s="476"/>
+      <c r="E20" s="482"/>
+      <c r="F20" s="483"/>
       <c r="G20" s="393"/>
       <c r="H20" s="393"/>
       <c r="I20" s="393"/>
@@ -6271,7 +6143,7 @@
       <c r="M26" s="416"/>
     </row>
     <row r="27" spans="2:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="424" t="s">
+      <c r="B27" s="422" t="s">
         <v>179</v>
       </c>
       <c r="C27" s="420"/>
@@ -6287,245 +6159,245 @@
       <c r="M27" s="416"/>
     </row>
     <row r="28" spans="2:22" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="492" t="s">
+      <c r="B28" s="487" t="s">
         <v>29</v>
       </c>
-      <c r="C28" s="493"/>
-      <c r="D28" s="494"/>
-      <c r="E28" s="495" t="s">
+      <c r="C28" s="488"/>
+      <c r="D28" s="489"/>
+      <c r="E28" s="490" t="s">
         <v>180</v>
       </c>
-      <c r="F28" s="495"/>
-      <c r="G28" s="495"/>
-      <c r="H28" s="495"/>
-      <c r="I28" s="495"/>
-      <c r="J28" s="495"/>
+      <c r="F28" s="490"/>
+      <c r="G28" s="490"/>
+      <c r="H28" s="490"/>
+      <c r="I28" s="490"/>
+      <c r="J28" s="490"/>
       <c r="K28" s="394"/>
-      <c r="L28" s="425"/>
-      <c r="M28" s="426"/>
-      <c r="N28" s="427"/>
+      <c r="L28" s="423"/>
+      <c r="M28" s="424"/>
+      <c r="N28" s="425"/>
       <c r="O28" s="412"/>
       <c r="P28" s="412"/>
-      <c r="Q28" s="425"/>
-      <c r="R28" s="425"/>
-      <c r="S28" s="425"/>
-      <c r="T28" s="496"/>
-      <c r="U28" s="496"/>
-      <c r="V28" s="496"/>
+      <c r="Q28" s="423"/>
+      <c r="R28" s="423"/>
+      <c r="S28" s="423"/>
+      <c r="T28" s="491"/>
+      <c r="U28" s="491"/>
+      <c r="V28" s="491"/>
     </row>
     <row r="29" spans="2:22" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="284" t="s">
         <v>27</v>
       </c>
-      <c r="C29" s="497" t="s">
+      <c r="C29" s="492" t="s">
         <v>28</v>
       </c>
-      <c r="D29" s="498"/>
-      <c r="E29" s="492">
+      <c r="D29" s="493"/>
+      <c r="E29" s="487">
         <v>1</v>
       </c>
-      <c r="F29" s="494"/>
-      <c r="G29" s="492">
+      <c r="F29" s="489"/>
+      <c r="G29" s="487">
         <v>2</v>
       </c>
-      <c r="H29" s="494"/>
-      <c r="I29" s="492">
+      <c r="H29" s="489"/>
+      <c r="I29" s="487">
         <v>3</v>
       </c>
-      <c r="J29" s="494"/>
+      <c r="J29" s="489"/>
       <c r="K29" s="395"/>
-      <c r="L29" s="425"/>
-      <c r="M29" s="426"/>
-      <c r="N29" s="427"/>
-      <c r="O29" s="425"/>
-      <c r="Q29" s="428"/>
-      <c r="S29" s="429"/>
-      <c r="T29" s="425"/>
-      <c r="U29" s="430"/>
+      <c r="L29" s="423"/>
+      <c r="M29" s="424"/>
+      <c r="N29" s="425"/>
+      <c r="O29" s="423"/>
+      <c r="Q29" s="426"/>
+      <c r="S29" s="427"/>
+      <c r="T29" s="423"/>
+      <c r="U29" s="428"/>
     </row>
     <row r="30" spans="2:22" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="431">
+      <c r="B30" s="429">
         <v>3</v>
       </c>
-      <c r="C30" s="488">
+      <c r="C30" s="494">
         <v>2.5</v>
       </c>
-      <c r="D30" s="489"/>
-      <c r="E30" s="490"/>
-      <c r="F30" s="491"/>
-      <c r="G30" s="490" t="s">
+      <c r="D30" s="495"/>
+      <c r="E30" s="496"/>
+      <c r="F30" s="497"/>
+      <c r="G30" s="496" t="s">
         <v>56</v>
       </c>
-      <c r="H30" s="491"/>
-      <c r="I30" s="490" t="s">
+      <c r="H30" s="497"/>
+      <c r="I30" s="496" t="s">
         <v>56</v>
       </c>
-      <c r="J30" s="491"/>
+      <c r="J30" s="497"/>
       <c r="K30" s="396"/>
-      <c r="L30" s="425"/>
-      <c r="M30" s="455"/>
-      <c r="N30" s="427"/>
-      <c r="O30" s="425"/>
-      <c r="Q30" s="432"/>
-      <c r="S30" s="429"/>
-      <c r="T30" s="425"/>
-      <c r="U30" s="430"/>
+      <c r="L30" s="423"/>
+      <c r="M30" s="453"/>
+      <c r="N30" s="425"/>
+      <c r="O30" s="423"/>
+      <c r="Q30" s="430"/>
+      <c r="S30" s="427"/>
+      <c r="T30" s="423"/>
+      <c r="U30" s="428"/>
     </row>
     <row r="31" spans="2:22" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="433">
+      <c r="B31" s="431">
         <v>2.5</v>
       </c>
-      <c r="C31" s="488">
+      <c r="C31" s="494">
         <v>2</v>
       </c>
-      <c r="D31" s="489"/>
-      <c r="E31" s="490"/>
-      <c r="F31" s="491"/>
-      <c r="G31" s="490" t="s">
+      <c r="D31" s="495"/>
+      <c r="E31" s="496"/>
+      <c r="F31" s="497"/>
+      <c r="G31" s="496" t="s">
         <v>56</v>
       </c>
-      <c r="H31" s="491"/>
-      <c r="I31" s="490" t="s">
+      <c r="H31" s="497"/>
+      <c r="I31" s="496" t="s">
         <v>56</v>
       </c>
-      <c r="J31" s="491"/>
+      <c r="J31" s="497"/>
       <c r="K31" s="396"/>
-      <c r="L31" s="434"/>
-      <c r="M31" s="426"/>
-      <c r="N31" s="427"/>
-      <c r="O31" s="434"/>
-      <c r="P31" s="434"/>
-      <c r="Q31" s="434"/>
-      <c r="R31" s="434"/>
-      <c r="S31" s="429"/>
-      <c r="T31" s="425"/>
-      <c r="U31" s="435"/>
+      <c r="L31" s="432"/>
+      <c r="M31" s="424"/>
+      <c r="N31" s="425"/>
+      <c r="O31" s="432"/>
+      <c r="P31" s="432"/>
+      <c r="Q31" s="432"/>
+      <c r="R31" s="432"/>
+      <c r="S31" s="427"/>
+      <c r="T31" s="423"/>
+      <c r="U31" s="433"/>
     </row>
     <row r="32" spans="2:22" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="431">
+      <c r="B32" s="429">
         <v>2</v>
       </c>
-      <c r="C32" s="488">
+      <c r="C32" s="494">
         <v>1.5</v>
       </c>
-      <c r="D32" s="489"/>
-      <c r="E32" s="490"/>
-      <c r="F32" s="491"/>
-      <c r="G32" s="490"/>
-      <c r="H32" s="491"/>
-      <c r="I32" s="490" t="s">
+      <c r="D32" s="495"/>
+      <c r="E32" s="496"/>
+      <c r="F32" s="497"/>
+      <c r="G32" s="496"/>
+      <c r="H32" s="497"/>
+      <c r="I32" s="496" t="s">
         <v>56</v>
       </c>
-      <c r="J32" s="491"/>
+      <c r="J32" s="497"/>
       <c r="K32" s="396"/>
-      <c r="L32" s="434"/>
-      <c r="M32" s="426"/>
-      <c r="N32" s="427"/>
-      <c r="O32" s="434"/>
-      <c r="P32" s="434"/>
-      <c r="Q32" s="434"/>
-      <c r="R32" s="434"/>
-      <c r="S32" s="434"/>
-      <c r="T32" s="434"/>
-      <c r="U32" s="434"/>
-      <c r="V32" s="434"/>
+      <c r="L32" s="432"/>
+      <c r="M32" s="424"/>
+      <c r="N32" s="425"/>
+      <c r="O32" s="432"/>
+      <c r="P32" s="432"/>
+      <c r="Q32" s="432"/>
+      <c r="R32" s="432"/>
+      <c r="S32" s="432"/>
+      <c r="T32" s="432"/>
+      <c r="U32" s="432"/>
+      <c r="V32" s="432"/>
     </row>
     <row r="33" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="433">
+      <c r="B33" s="431">
         <v>1.5</v>
       </c>
-      <c r="C33" s="488">
+      <c r="C33" s="494">
         <v>1</v>
       </c>
-      <c r="D33" s="489"/>
-      <c r="E33" s="490" t="s">
+      <c r="D33" s="495"/>
+      <c r="E33" s="496" t="s">
         <v>56</v>
       </c>
-      <c r="F33" s="491"/>
-      <c r="G33" s="490"/>
-      <c r="H33" s="491"/>
-      <c r="I33" s="490"/>
-      <c r="J33" s="491"/>
+      <c r="F33" s="497"/>
+      <c r="G33" s="496"/>
+      <c r="H33" s="497"/>
+      <c r="I33" s="496"/>
+      <c r="J33" s="497"/>
       <c r="K33" s="396"/>
-      <c r="L33" s="436"/>
-      <c r="M33" s="426"/>
-      <c r="N33" s="427"/>
-      <c r="O33" s="486"/>
-      <c r="P33" s="486"/>
-      <c r="Q33" s="486"/>
-      <c r="R33" s="437"/>
-      <c r="S33" s="437"/>
-      <c r="T33" s="486"/>
-      <c r="U33" s="486"/>
-      <c r="V33" s="437"/>
-      <c r="W33" s="487"/>
-      <c r="X33" s="487"/>
-      <c r="Y33" s="487"/>
+      <c r="L33" s="434"/>
+      <c r="M33" s="424"/>
+      <c r="N33" s="425"/>
+      <c r="O33" s="498"/>
+      <c r="P33" s="498"/>
+      <c r="Q33" s="498"/>
+      <c r="R33" s="435"/>
+      <c r="S33" s="435"/>
+      <c r="T33" s="498"/>
+      <c r="U33" s="498"/>
+      <c r="V33" s="435"/>
+      <c r="W33" s="499"/>
+      <c r="X33" s="499"/>
+      <c r="Y33" s="499"/>
     </row>
     <row r="34" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="431">
+      <c r="B34" s="429">
         <v>1</v>
       </c>
-      <c r="C34" s="488">
+      <c r="C34" s="494">
         <v>0.75</v>
       </c>
-      <c r="D34" s="489"/>
-      <c r="E34" s="490" t="s">
+      <c r="D34" s="495"/>
+      <c r="E34" s="496" t="s">
         <v>56</v>
       </c>
-      <c r="F34" s="491"/>
-      <c r="G34" s="490" t="s">
+      <c r="F34" s="497"/>
+      <c r="G34" s="496" t="s">
         <v>56</v>
       </c>
-      <c r="H34" s="491"/>
-      <c r="I34" s="490"/>
-      <c r="J34" s="491"/>
+      <c r="H34" s="497"/>
+      <c r="I34" s="496"/>
+      <c r="J34" s="497"/>
       <c r="K34" s="396"/>
-      <c r="L34" s="436"/>
-      <c r="M34" s="426"/>
-      <c r="N34" s="427"/>
-      <c r="O34" s="437"/>
-      <c r="P34" s="437"/>
-      <c r="Q34" s="437"/>
-      <c r="R34" s="437"/>
-      <c r="S34" s="437"/>
-      <c r="T34" s="437"/>
-      <c r="U34" s="437"/>
-      <c r="V34" s="437"/>
-      <c r="W34" s="487"/>
-      <c r="X34" s="487"/>
-      <c r="Y34" s="487"/>
+      <c r="L34" s="434"/>
+      <c r="M34" s="424"/>
+      <c r="N34" s="425"/>
+      <c r="O34" s="435"/>
+      <c r="P34" s="435"/>
+      <c r="Q34" s="435"/>
+      <c r="R34" s="435"/>
+      <c r="S34" s="435"/>
+      <c r="T34" s="435"/>
+      <c r="U34" s="435"/>
+      <c r="V34" s="435"/>
+      <c r="W34" s="499"/>
+      <c r="X34" s="499"/>
+      <c r="Y34" s="499"/>
     </row>
     <row r="35" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="467" t="s">
+      <c r="B35" s="500" t="s">
         <v>181</v>
       </c>
-      <c r="C35" s="480"/>
-      <c r="D35" s="468"/>
-      <c r="E35" s="467"/>
-      <c r="F35" s="468"/>
-      <c r="G35" s="467"/>
-      <c r="H35" s="468"/>
-      <c r="I35" s="467"/>
-      <c r="J35" s="468"/>
+      <c r="C35" s="501"/>
+      <c r="D35" s="502"/>
+      <c r="E35" s="500"/>
+      <c r="F35" s="502"/>
+      <c r="G35" s="500"/>
+      <c r="H35" s="502"/>
+      <c r="I35" s="500"/>
+      <c r="J35" s="502"/>
       <c r="K35" s="396"/>
-      <c r="L35" s="436"/>
-      <c r="M35" s="426"/>
-      <c r="N35" s="427"/>
-      <c r="O35" s="437"/>
-      <c r="P35" s="437"/>
-      <c r="Q35" s="437"/>
-      <c r="R35" s="437"/>
-      <c r="S35" s="437"/>
-      <c r="T35" s="437"/>
-      <c r="U35" s="437"/>
-      <c r="V35" s="437"/>
-      <c r="W35" s="438"/>
-      <c r="X35" s="438"/>
-      <c r="Y35" s="438"/>
+      <c r="L35" s="434"/>
+      <c r="M35" s="424"/>
+      <c r="N35" s="425"/>
+      <c r="O35" s="435"/>
+      <c r="P35" s="435"/>
+      <c r="Q35" s="435"/>
+      <c r="R35" s="435"/>
+      <c r="S35" s="435"/>
+      <c r="T35" s="435"/>
+      <c r="U35" s="435"/>
+      <c r="V35" s="435"/>
+      <c r="W35" s="436"/>
+      <c r="X35" s="436"/>
+      <c r="Y35" s="436"/>
     </row>
     <row r="36" spans="1:25" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="426"/>
+      <c r="B36" s="424"/>
       <c r="C36" s="397"/>
       <c r="D36" s="398"/>
       <c r="E36" s="398"/>
@@ -6535,186 +6407,186 @@
       <c r="I36" s="398"/>
       <c r="J36" s="398"/>
       <c r="K36" s="396"/>
-      <c r="L36" s="432"/>
-      <c r="M36" s="426"/>
-      <c r="N36" s="427"/>
-      <c r="O36" s="439"/>
-      <c r="Q36" s="440"/>
-      <c r="R36" s="428"/>
-      <c r="S36" s="432"/>
-      <c r="U36" s="432"/>
-      <c r="V36" s="432"/>
-      <c r="W36" s="432"/>
-      <c r="X36" s="432"/>
-      <c r="Y36" s="432"/>
+      <c r="L36" s="430"/>
+      <c r="M36" s="424"/>
+      <c r="N36" s="425"/>
+      <c r="O36" s="437"/>
+      <c r="Q36" s="438"/>
+      <c r="R36" s="426"/>
+      <c r="S36" s="430"/>
+      <c r="U36" s="430"/>
+      <c r="V36" s="430"/>
+      <c r="W36" s="430"/>
+      <c r="X36" s="430"/>
+      <c r="Y36" s="430"/>
     </row>
     <row r="37" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="441" t="s">
+      <c r="A37" s="439" t="s">
         <v>77</v>
       </c>
-      <c r="B37" s="481" t="s">
+      <c r="B37" s="474" t="s">
         <v>51</v>
       </c>
-      <c r="C37" s="482"/>
+      <c r="C37" s="475"/>
       <c r="D37" s="284" t="s">
         <v>38</v>
       </c>
-      <c r="E37" s="483" t="s">
+      <c r="E37" s="476" t="s">
         <v>182</v>
       </c>
-      <c r="F37" s="484"/>
-      <c r="G37" s="483" t="s">
+      <c r="F37" s="477"/>
+      <c r="G37" s="476" t="s">
         <v>183</v>
       </c>
-      <c r="H37" s="484"/>
-      <c r="I37" s="485" t="s">
+      <c r="H37" s="477"/>
+      <c r="I37" s="503" t="s">
         <v>184</v>
       </c>
-      <c r="J37" s="485"/>
+      <c r="J37" s="503"/>
       <c r="K37" s="396"/>
-      <c r="L37" s="442"/>
-      <c r="M37" s="426"/>
-      <c r="N37" s="427"/>
-      <c r="O37" s="443"/>
-      <c r="Q37" s="440"/>
-      <c r="R37" s="428"/>
-      <c r="S37" s="432"/>
-      <c r="U37" s="432"/>
-      <c r="V37" s="432"/>
-      <c r="W37" s="436"/>
-      <c r="X37" s="436"/>
-      <c r="Y37" s="436"/>
+      <c r="L37" s="440"/>
+      <c r="M37" s="424"/>
+      <c r="N37" s="425"/>
+      <c r="O37" s="441"/>
+      <c r="Q37" s="438"/>
+      <c r="R37" s="426"/>
+      <c r="S37" s="430"/>
+      <c r="U37" s="430"/>
+      <c r="V37" s="430"/>
+      <c r="W37" s="434"/>
+      <c r="X37" s="434"/>
+      <c r="Y37" s="434"/>
     </row>
     <row r="38" spans="1:25" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="431" t="s">
+      <c r="A38" s="429" t="s">
         <v>129</v>
       </c>
-      <c r="B38" s="478" t="s">
+      <c r="B38" s="480" t="s">
         <v>144</v>
       </c>
-      <c r="C38" s="479"/>
+      <c r="C38" s="481"/>
       <c r="D38" s="61" t="s">
         <v>39</v>
       </c>
-      <c r="E38" s="475"/>
-      <c r="F38" s="476"/>
-      <c r="G38" s="475"/>
-      <c r="H38" s="476"/>
-      <c r="I38" s="475"/>
-      <c r="J38" s="476"/>
+      <c r="E38" s="482"/>
+      <c r="F38" s="483"/>
+      <c r="G38" s="482"/>
+      <c r="H38" s="483"/>
+      <c r="I38" s="482"/>
+      <c r="J38" s="483"/>
       <c r="K38" s="396"/>
-      <c r="L38" s="442"/>
-      <c r="M38" s="426"/>
-      <c r="N38" s="427"/>
-      <c r="O38" s="443"/>
-      <c r="Q38" s="440"/>
-      <c r="R38" s="428"/>
-      <c r="S38" s="432"/>
-      <c r="U38" s="432"/>
-      <c r="V38" s="432"/>
-      <c r="W38" s="436"/>
-      <c r="X38" s="436"/>
-      <c r="Y38" s="436"/>
+      <c r="L38" s="440"/>
+      <c r="M38" s="424"/>
+      <c r="N38" s="425"/>
+      <c r="O38" s="441"/>
+      <c r="Q38" s="438"/>
+      <c r="R38" s="426"/>
+      <c r="S38" s="430"/>
+      <c r="U38" s="430"/>
+      <c r="V38" s="430"/>
+      <c r="W38" s="434"/>
+      <c r="X38" s="434"/>
+      <c r="Y38" s="434"/>
     </row>
     <row r="39" spans="1:25" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="431" t="s">
+      <c r="A39" s="429" t="s">
         <v>62</v>
       </c>
-      <c r="B39" s="473" t="s">
+      <c r="B39" s="504" t="s">
         <v>146</v>
       </c>
-      <c r="C39" s="474"/>
+      <c r="C39" s="505"/>
       <c r="D39" s="64" t="s">
         <v>39</v>
       </c>
-      <c r="E39" s="475"/>
-      <c r="F39" s="476"/>
-      <c r="G39" s="475"/>
-      <c r="H39" s="476"/>
-      <c r="I39" s="475"/>
-      <c r="J39" s="476"/>
+      <c r="E39" s="482"/>
+      <c r="F39" s="483"/>
+      <c r="G39" s="482"/>
+      <c r="H39" s="483"/>
+      <c r="I39" s="482"/>
+      <c r="J39" s="483"/>
       <c r="K39" s="396"/>
-      <c r="L39" s="442"/>
-      <c r="M39" s="426"/>
-      <c r="N39" s="427"/>
-      <c r="O39" s="443"/>
-      <c r="Q39" s="440"/>
-      <c r="R39" s="428"/>
-      <c r="S39" s="432"/>
-      <c r="U39" s="432"/>
-      <c r="V39" s="432"/>
-      <c r="W39" s="436"/>
-      <c r="X39" s="436"/>
-      <c r="Y39" s="436"/>
+      <c r="L39" s="440"/>
+      <c r="M39" s="424"/>
+      <c r="N39" s="425"/>
+      <c r="O39" s="441"/>
+      <c r="Q39" s="438"/>
+      <c r="R39" s="426"/>
+      <c r="S39" s="430"/>
+      <c r="U39" s="430"/>
+      <c r="V39" s="430"/>
+      <c r="W39" s="434"/>
+      <c r="X39" s="434"/>
+      <c r="Y39" s="434"/>
     </row>
     <row r="40" spans="1:25" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="61" t="s">
         <v>63</v>
       </c>
-      <c r="B40" s="473" t="s">
+      <c r="B40" s="504" t="s">
         <v>185</v>
       </c>
-      <c r="C40" s="474"/>
+      <c r="C40" s="505"/>
       <c r="D40" s="64" t="s">
         <v>39</v>
       </c>
-      <c r="E40" s="475"/>
-      <c r="F40" s="476"/>
-      <c r="G40" s="475"/>
-      <c r="H40" s="476"/>
-      <c r="I40" s="475"/>
-      <c r="J40" s="476"/>
+      <c r="E40" s="482"/>
+      <c r="F40" s="483"/>
+      <c r="G40" s="482"/>
+      <c r="H40" s="483"/>
+      <c r="I40" s="482"/>
+      <c r="J40" s="483"/>
       <c r="K40" s="399"/>
-      <c r="M40" s="426"/>
-      <c r="N40" s="427"/>
-      <c r="O40" s="439"/>
-      <c r="Q40" s="440"/>
-      <c r="R40" s="428"/>
-      <c r="S40" s="432"/>
-      <c r="U40" s="432"/>
-      <c r="V40" s="432"/>
-      <c r="W40" s="432"/>
-      <c r="X40" s="444"/>
-      <c r="Y40" s="432"/>
+      <c r="M40" s="424"/>
+      <c r="N40" s="425"/>
+      <c r="O40" s="437"/>
+      <c r="Q40" s="438"/>
+      <c r="R40" s="426"/>
+      <c r="S40" s="430"/>
+      <c r="U40" s="430"/>
+      <c r="V40" s="430"/>
+      <c r="W40" s="430"/>
+      <c r="X40" s="442"/>
+      <c r="Y40" s="430"/>
     </row>
     <row r="41" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="61" t="s">
         <v>64</v>
       </c>
-      <c r="B41" s="473" t="s">
+      <c r="B41" s="504" t="s">
         <v>186</v>
       </c>
-      <c r="C41" s="474"/>
+      <c r="C41" s="505"/>
       <c r="D41" s="64" t="s">
         <v>39</v>
       </c>
-      <c r="E41" s="475"/>
-      <c r="F41" s="476"/>
-      <c r="G41" s="475"/>
-      <c r="H41" s="476"/>
-      <c r="I41" s="475"/>
-      <c r="J41" s="476"/>
+      <c r="E41" s="482"/>
+      <c r="F41" s="483"/>
+      <c r="G41" s="482"/>
+      <c r="H41" s="483"/>
+      <c r="I41" s="482"/>
+      <c r="J41" s="483"/>
       <c r="K41" s="399"/>
-      <c r="M41" s="426"/>
-      <c r="N41" s="427"/>
-      <c r="O41" s="439"/>
-      <c r="Q41" s="440"/>
-      <c r="R41" s="428"/>
-      <c r="S41" s="432"/>
-      <c r="U41" s="432"/>
-      <c r="V41" s="432"/>
-      <c r="W41" s="432"/>
-      <c r="X41" s="444"/>
-      <c r="Y41" s="432"/>
+      <c r="M41" s="424"/>
+      <c r="N41" s="425"/>
+      <c r="O41" s="437"/>
+      <c r="Q41" s="438"/>
+      <c r="R41" s="426"/>
+      <c r="S41" s="430"/>
+      <c r="U41" s="430"/>
+      <c r="V41" s="430"/>
+      <c r="W41" s="430"/>
+      <c r="X41" s="442"/>
+      <c r="Y41" s="430"/>
     </row>
     <row r="42" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="61" t="s">
         <v>65</v>
       </c>
-      <c r="B42" s="473" t="s">
+      <c r="B42" s="504" t="s">
         <v>187</v>
       </c>
-      <c r="C42" s="474"/>
+      <c r="C42" s="505"/>
       <c r="D42" s="64" t="s">
         <v>39</v>
       </c>
@@ -6725,243 +6597,243 @@
       <c r="I42" s="400"/>
       <c r="J42" s="401"/>
       <c r="K42" s="399"/>
-      <c r="M42" s="426"/>
-      <c r="N42" s="427"/>
-      <c r="O42" s="439"/>
-      <c r="Q42" s="440"/>
-      <c r="R42" s="428"/>
-      <c r="S42" s="432"/>
-      <c r="U42" s="432"/>
-      <c r="V42" s="432"/>
-      <c r="W42" s="432"/>
-      <c r="X42" s="444"/>
-      <c r="Y42" s="432"/>
+      <c r="M42" s="424"/>
+      <c r="N42" s="425"/>
+      <c r="O42" s="437"/>
+      <c r="Q42" s="438"/>
+      <c r="R42" s="426"/>
+      <c r="S42" s="430"/>
+      <c r="U42" s="430"/>
+      <c r="V42" s="430"/>
+      <c r="W42" s="430"/>
+      <c r="X42" s="442"/>
+      <c r="Y42" s="430"/>
     </row>
     <row r="43" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="61" t="s">
         <v>130</v>
       </c>
-      <c r="B43" s="473" t="s">
+      <c r="B43" s="504" t="s">
         <v>141</v>
       </c>
-      <c r="C43" s="474"/>
+      <c r="C43" s="505"/>
       <c r="D43" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="E43" s="475"/>
-      <c r="F43" s="476"/>
-      <c r="G43" s="475"/>
-      <c r="H43" s="476"/>
-      <c r="I43" s="475"/>
-      <c r="J43" s="476"/>
+      <c r="E43" s="482"/>
+      <c r="F43" s="483"/>
+      <c r="G43" s="482"/>
+      <c r="H43" s="483"/>
+      <c r="I43" s="482"/>
+      <c r="J43" s="483"/>
       <c r="K43" s="402"/>
-      <c r="M43" s="445"/>
-      <c r="N43" s="427"/>
-      <c r="O43" s="443"/>
-      <c r="Q43" s="440"/>
-      <c r="R43" s="428"/>
-      <c r="S43" s="432"/>
-      <c r="U43" s="432"/>
-      <c r="V43" s="432"/>
-      <c r="W43" s="446"/>
-      <c r="X43" s="447"/>
-      <c r="Y43" s="446"/>
+      <c r="M43" s="443"/>
+      <c r="N43" s="425"/>
+      <c r="O43" s="441"/>
+      <c r="Q43" s="438"/>
+      <c r="R43" s="426"/>
+      <c r="S43" s="430"/>
+      <c r="U43" s="430"/>
+      <c r="V43" s="430"/>
+      <c r="W43" s="444"/>
+      <c r="X43" s="445"/>
+      <c r="Y43" s="444"/>
     </row>
     <row r="44" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="61"/>
-      <c r="B44" s="473" t="s">
+      <c r="B44" s="504" t="s">
         <v>188</v>
       </c>
-      <c r="C44" s="477"/>
+      <c r="C44" s="506"/>
       <c r="D44" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="E44" s="475"/>
-      <c r="F44" s="476"/>
-      <c r="G44" s="475"/>
-      <c r="H44" s="476"/>
-      <c r="I44" s="475"/>
-      <c r="J44" s="476"/>
+      <c r="E44" s="482"/>
+      <c r="F44" s="483"/>
+      <c r="G44" s="482"/>
+      <c r="H44" s="483"/>
+      <c r="I44" s="482"/>
+      <c r="J44" s="483"/>
       <c r="K44" s="402"/>
-      <c r="M44" s="445"/>
-      <c r="N44" s="427"/>
-      <c r="O44" s="443"/>
-      <c r="Q44" s="440"/>
-      <c r="R44" s="428"/>
-      <c r="S44" s="432"/>
-      <c r="U44" s="432"/>
-      <c r="V44" s="432"/>
-      <c r="W44" s="446"/>
-      <c r="X44" s="447"/>
-      <c r="Y44" s="446"/>
+      <c r="M44" s="443"/>
+      <c r="N44" s="425"/>
+      <c r="O44" s="441"/>
+      <c r="Q44" s="438"/>
+      <c r="R44" s="426"/>
+      <c r="S44" s="430"/>
+      <c r="U44" s="430"/>
+      <c r="V44" s="430"/>
+      <c r="W44" s="444"/>
+      <c r="X44" s="445"/>
+      <c r="Y44" s="444"/>
     </row>
     <row r="45" spans="1:25" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="448"/>
-      <c r="C45" s="448"/>
-      <c r="D45" s="448"/>
-      <c r="E45" s="448"/>
-      <c r="F45" s="448"/>
+      <c r="B45" s="446"/>
+      <c r="C45" s="446"/>
+      <c r="D45" s="446"/>
+      <c r="E45" s="446"/>
+      <c r="F45" s="446"/>
       <c r="M45" s="416"/>
-      <c r="N45" s="427"/>
-      <c r="O45" s="443"/>
-      <c r="Q45" s="440"/>
-      <c r="R45" s="428"/>
-      <c r="S45" s="432"/>
-      <c r="U45" s="432"/>
-      <c r="V45" s="432"/>
-      <c r="W45" s="446"/>
-      <c r="X45" s="447"/>
-      <c r="Y45" s="446"/>
+      <c r="N45" s="425"/>
+      <c r="O45" s="441"/>
+      <c r="Q45" s="438"/>
+      <c r="R45" s="426"/>
+      <c r="S45" s="430"/>
+      <c r="U45" s="430"/>
+      <c r="V45" s="430"/>
+      <c r="W45" s="444"/>
+      <c r="X45" s="445"/>
+      <c r="Y45" s="444"/>
     </row>
     <row r="46" spans="1:25" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="469" t="s">
+      <c r="B46" s="509" t="s">
         <v>189</v>
       </c>
-      <c r="C46" s="470" t="s">
+      <c r="C46" s="510" t="s">
         <v>190</v>
       </c>
-      <c r="D46" s="470"/>
-      <c r="E46" s="469"/>
-      <c r="F46" s="469"/>
-      <c r="G46" s="470" t="s">
+      <c r="D46" s="510"/>
+      <c r="E46" s="509"/>
+      <c r="F46" s="509"/>
+      <c r="G46" s="510" t="s">
         <v>191</v>
       </c>
-      <c r="H46" s="470"/>
-      <c r="I46" s="471"/>
-      <c r="J46" s="471"/>
+      <c r="H46" s="510"/>
+      <c r="I46" s="511"/>
+      <c r="J46" s="511"/>
       <c r="M46" s="416"/>
-      <c r="N46" s="427"/>
-      <c r="O46" s="439"/>
-      <c r="Q46" s="440"/>
-      <c r="R46" s="428"/>
-      <c r="S46" s="432"/>
-      <c r="U46" s="432"/>
-      <c r="V46" s="432"/>
-      <c r="W46" s="446"/>
-      <c r="X46" s="447"/>
-      <c r="Y46" s="446"/>
+      <c r="N46" s="425"/>
+      <c r="O46" s="437"/>
+      <c r="Q46" s="438"/>
+      <c r="R46" s="426"/>
+      <c r="S46" s="430"/>
+      <c r="U46" s="430"/>
+      <c r="V46" s="430"/>
+      <c r="W46" s="444"/>
+      <c r="X46" s="445"/>
+      <c r="Y46" s="444"/>
     </row>
     <row r="47" spans="1:25" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="469"/>
-      <c r="C47" s="470" t="s">
+      <c r="B47" s="509"/>
+      <c r="C47" s="510" t="s">
         <v>192</v>
       </c>
-      <c r="D47" s="470"/>
-      <c r="E47" s="470"/>
-      <c r="F47" s="470"/>
-      <c r="G47" s="470" t="s">
+      <c r="D47" s="510"/>
+      <c r="E47" s="510"/>
+      <c r="F47" s="510"/>
+      <c r="G47" s="510" t="s">
         <v>193</v>
       </c>
-      <c r="H47" s="470"/>
-      <c r="I47" s="472"/>
-      <c r="J47" s="472"/>
+      <c r="H47" s="510"/>
+      <c r="I47" s="512"/>
+      <c r="J47" s="512"/>
       <c r="M47" s="416"/>
-      <c r="N47" s="427"/>
-      <c r="O47" s="439"/>
-      <c r="Q47" s="440"/>
-      <c r="R47" s="428"/>
-      <c r="S47" s="432"/>
-      <c r="U47" s="432"/>
-      <c r="V47" s="432"/>
-      <c r="W47" s="446"/>
-      <c r="X47" s="447"/>
-      <c r="Y47" s="446"/>
+      <c r="N47" s="425"/>
+      <c r="O47" s="437"/>
+      <c r="Q47" s="438"/>
+      <c r="R47" s="426"/>
+      <c r="S47" s="430"/>
+      <c r="U47" s="430"/>
+      <c r="V47" s="430"/>
+      <c r="W47" s="444"/>
+      <c r="X47" s="445"/>
+      <c r="Y47" s="444"/>
     </row>
     <row r="48" spans="1:25" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="403"/>
       <c r="M48" s="416"/>
-      <c r="N48" s="427"/>
-      <c r="O48" s="439"/>
-      <c r="Q48" s="440"/>
-      <c r="R48" s="428"/>
-      <c r="S48" s="432"/>
-      <c r="U48" s="432"/>
-      <c r="V48" s="432"/>
-      <c r="W48" s="446"/>
-      <c r="X48" s="447"/>
-      <c r="Y48" s="446"/>
+      <c r="N48" s="425"/>
+      <c r="O48" s="437"/>
+      <c r="Q48" s="438"/>
+      <c r="R48" s="426"/>
+      <c r="S48" s="430"/>
+      <c r="U48" s="430"/>
+      <c r="V48" s="430"/>
+      <c r="W48" s="444"/>
+      <c r="X48" s="445"/>
+      <c r="Y48" s="444"/>
     </row>
     <row r="49" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="449" t="s">
+      <c r="A49" s="447" t="s">
         <v>57</v>
       </c>
-      <c r="B49" s="450"/>
-      <c r="C49" s="450"/>
-      <c r="D49" s="450"/>
-      <c r="E49" s="450"/>
-      <c r="F49" s="450"/>
-      <c r="G49" s="450"/>
-      <c r="H49" s="450"/>
-      <c r="I49" s="450"/>
-      <c r="J49" s="450"/>
+      <c r="B49" s="448"/>
+      <c r="C49" s="448"/>
+      <c r="D49" s="448"/>
+      <c r="E49" s="448"/>
+      <c r="F49" s="448"/>
+      <c r="G49" s="448"/>
+      <c r="H49" s="448"/>
+      <c r="I49" s="448"/>
+      <c r="J49" s="448"/>
       <c r="M49" s="416"/>
-      <c r="N49" s="427"/>
-      <c r="O49" s="439"/>
-      <c r="Q49" s="440"/>
-      <c r="R49" s="428"/>
-      <c r="S49" s="432"/>
-      <c r="U49" s="432"/>
-      <c r="V49" s="432"/>
-      <c r="W49" s="446"/>
-      <c r="X49" s="447"/>
-      <c r="Y49" s="446"/>
+      <c r="N49" s="425"/>
+      <c r="O49" s="437"/>
+      <c r="Q49" s="438"/>
+      <c r="R49" s="426"/>
+      <c r="S49" s="430"/>
+      <c r="U49" s="430"/>
+      <c r="V49" s="430"/>
+      <c r="W49" s="444"/>
+      <c r="X49" s="445"/>
+      <c r="Y49" s="444"/>
     </row>
     <row r="50" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C50" s="451"/>
-      <c r="D50" s="451"/>
-      <c r="E50" s="451"/>
-      <c r="F50" s="451"/>
-      <c r="G50" s="451"/>
-      <c r="H50" s="451"/>
-      <c r="I50" s="451"/>
-      <c r="J50" s="451"/>
+      <c r="C50" s="449"/>
+      <c r="D50" s="449"/>
+      <c r="E50" s="449"/>
+      <c r="F50" s="449"/>
+      <c r="G50" s="449"/>
+      <c r="H50" s="449"/>
+      <c r="I50" s="449"/>
+      <c r="J50" s="449"/>
       <c r="M50" s="416"/>
-      <c r="N50" s="452"/>
-      <c r="O50" s="439"/>
-      <c r="Q50" s="440"/>
-      <c r="R50" s="428"/>
-      <c r="S50" s="432"/>
-      <c r="U50" s="432"/>
-      <c r="V50" s="432"/>
-      <c r="W50" s="446"/>
-      <c r="X50" s="447"/>
-      <c r="Y50" s="446"/>
+      <c r="N50" s="450"/>
+      <c r="O50" s="437"/>
+      <c r="Q50" s="438"/>
+      <c r="R50" s="426"/>
+      <c r="S50" s="430"/>
+      <c r="U50" s="430"/>
+      <c r="V50" s="430"/>
+      <c r="W50" s="444"/>
+      <c r="X50" s="445"/>
+      <c r="Y50" s="444"/>
     </row>
     <row r="51" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D51" s="451"/>
-      <c r="E51" s="451"/>
-      <c r="F51" s="451"/>
-      <c r="G51" s="451"/>
+      <c r="D51" s="449"/>
+      <c r="E51" s="449"/>
+      <c r="F51" s="449"/>
+      <c r="G51" s="449"/>
       <c r="M51" s="416"/>
-      <c r="O51" s="439"/>
-      <c r="Q51" s="440"/>
-      <c r="R51" s="428"/>
-      <c r="S51" s="432"/>
-      <c r="U51" s="432"/>
-      <c r="V51" s="432"/>
-      <c r="W51" s="432"/>
-      <c r="X51" s="453"/>
-      <c r="Y51" s="432"/>
+      <c r="O51" s="437"/>
+      <c r="Q51" s="438"/>
+      <c r="R51" s="426"/>
+      <c r="S51" s="430"/>
+      <c r="U51" s="430"/>
+      <c r="V51" s="430"/>
+      <c r="W51" s="430"/>
+      <c r="X51" s="451"/>
+      <c r="Y51" s="430"/>
     </row>
     <row r="52" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="406" t="s">
         <v>194</v>
       </c>
-      <c r="C52" s="451"/>
-      <c r="D52" s="451"/>
-      <c r="E52" s="451"/>
-      <c r="F52" s="451"/>
-      <c r="G52" s="451"/>
-      <c r="H52" s="451"/>
-      <c r="I52" s="451"/>
-      <c r="J52" s="451"/>
+      <c r="C52" s="449"/>
+      <c r="D52" s="449"/>
+      <c r="E52" s="449"/>
+      <c r="F52" s="449"/>
+      <c r="G52" s="449"/>
+      <c r="H52" s="449"/>
+      <c r="I52" s="449"/>
+      <c r="J52" s="449"/>
       <c r="M52" s="416"/>
-      <c r="O52" s="439"/>
-      <c r="Q52" s="440"/>
-      <c r="R52" s="428"/>
-      <c r="S52" s="432"/>
-      <c r="U52" s="432"/>
-      <c r="V52" s="432"/>
+      <c r="O52" s="437"/>
+      <c r="Q52" s="438"/>
+      <c r="R52" s="426"/>
+      <c r="S52" s="430"/>
+      <c r="U52" s="430"/>
+      <c r="V52" s="430"/>
     </row>
     <row r="53" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C53" s="413"/>
@@ -6973,19 +6845,19 @@
       <c r="I53" s="413"/>
       <c r="J53" s="413"/>
       <c r="M53" s="416"/>
-      <c r="O53" s="429"/>
-      <c r="Q53" s="429"/>
-      <c r="R53" s="432"/>
-      <c r="S53" s="432"/>
-      <c r="U53" s="432"/>
-      <c r="V53" s="429"/>
+      <c r="O53" s="427"/>
+      <c r="Q53" s="427"/>
+      <c r="R53" s="430"/>
+      <c r="S53" s="430"/>
+      <c r="U53" s="430"/>
+      <c r="V53" s="427"/>
     </row>
     <row r="54" spans="1:25" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="403" t="s">
         <v>20</v>
       </c>
       <c r="B54" s="403"/>
-      <c r="L54" s="432"/>
+      <c r="L54" s="430"/>
       <c r="M54" s="416"/>
     </row>
     <row r="55" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -6993,34 +6865,34 @@
         <v>195</v>
       </c>
       <c r="B55" s="403"/>
-      <c r="C55" s="454"/>
-      <c r="D55" s="454"/>
-      <c r="E55" s="454"/>
-      <c r="F55" s="454"/>
-      <c r="G55" s="454"/>
-      <c r="H55" s="454"/>
-      <c r="I55" s="454"/>
-      <c r="J55" s="454"/>
-      <c r="K55" s="454"/>
+      <c r="C55" s="452"/>
+      <c r="D55" s="452"/>
+      <c r="E55" s="452"/>
+      <c r="F55" s="452"/>
+      <c r="G55" s="452"/>
+      <c r="H55" s="452"/>
+      <c r="I55" s="452"/>
+      <c r="J55" s="452"/>
+      <c r="K55" s="452"/>
       <c r="L55" s="416"/>
       <c r="M55" s="416"/>
       <c r="N55" s="416"/>
     </row>
     <row r="56" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="57" spans="1:25" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="465" t="s">
+      <c r="A57" s="507" t="s">
         <v>196</v>
       </c>
-      <c r="B57" s="465"/>
-      <c r="C57" s="465"/>
-      <c r="D57" s="465"/>
-      <c r="E57" s="465"/>
-      <c r="F57" s="465"/>
-      <c r="G57" s="465"/>
-      <c r="H57" s="465"/>
-      <c r="I57" s="465"/>
-      <c r="J57" s="465"/>
-      <c r="K57" s="465"/>
+      <c r="B57" s="507"/>
+      <c r="C57" s="507"/>
+      <c r="D57" s="507"/>
+      <c r="E57" s="507"/>
+      <c r="F57" s="507"/>
+      <c r="G57" s="507"/>
+      <c r="H57" s="507"/>
+      <c r="I57" s="507"/>
+      <c r="J57" s="507"/>
+      <c r="K57" s="507"/>
     </row>
     <row r="58" spans="1:25" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="59" spans="1:25" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -7031,72 +6903,23 @@
     <protectedRange sqref="T8:T9" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="99">
-    <mergeCell ref="A7:K7"/>
-    <mergeCell ref="A8:K8"/>
-    <mergeCell ref="S8:U8"/>
-    <mergeCell ref="V8:W8"/>
-    <mergeCell ref="S9:U9"/>
-    <mergeCell ref="V9:W9"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="A13:K13"/>
-    <mergeCell ref="A14:K14"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="E28:J28"/>
-    <mergeCell ref="T28:V28"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="G33:H33"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="O33:Q33"/>
-    <mergeCell ref="T33:U33"/>
-    <mergeCell ref="W33:Y34"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="G34:H34"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="G35:H35"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="I37:J37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="G39:H39"/>
-    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="I43:J43"/>
+    <mergeCell ref="A57:K57"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="G47:H47"/>
     <mergeCell ref="B44:C44"/>
     <mergeCell ref="E44:F44"/>
     <mergeCell ref="G44:H44"/>
@@ -7113,23 +6936,72 @@
     <mergeCell ref="B43:C43"/>
     <mergeCell ref="E43:F43"/>
     <mergeCell ref="G43:H43"/>
-    <mergeCell ref="I43:J43"/>
-    <mergeCell ref="A57:K57"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="E46:F46"/>
-    <mergeCell ref="G46:H46"/>
-    <mergeCell ref="I46:J46"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="G47:H47"/>
-    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="G39:H39"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="G35:H35"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="O33:Q33"/>
+    <mergeCell ref="T33:U33"/>
+    <mergeCell ref="W33:Y34"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="G34:H34"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="G33:H33"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="E28:J28"/>
+    <mergeCell ref="T28:V28"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="A13:K13"/>
+    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="A7:K7"/>
+    <mergeCell ref="A8:K8"/>
+    <mergeCell ref="S8:U8"/>
+    <mergeCell ref="V8:W8"/>
+    <mergeCell ref="S9:U9"/>
+    <mergeCell ref="V9:W9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7167,16 +7039,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="515"/>
-      <c r="B1" s="515"/>
-      <c r="C1" s="515"/>
-      <c r="D1" s="515"/>
-      <c r="E1" s="515"/>
-      <c r="F1" s="515"/>
-      <c r="G1" s="515"/>
-      <c r="H1" s="515"/>
-      <c r="I1" s="515"/>
-      <c r="J1" s="515"/>
+      <c r="A1" s="523"/>
+      <c r="B1" s="523"/>
+      <c r="C1" s="523"/>
+      <c r="D1" s="523"/>
+      <c r="E1" s="523"/>
+      <c r="F1" s="523"/>
+      <c r="G1" s="523"/>
+      <c r="H1" s="523"/>
+      <c r="I1" s="523"/>
+      <c r="J1" s="523"/>
     </row>
     <row r="2" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="93"/>
@@ -7227,34 +7099,34 @@
       <c r="J5" s="93"/>
     </row>
     <row r="6" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="515" t="s">
+      <c r="A6" s="523" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="515"/>
-      <c r="C6" s="515"/>
-      <c r="D6" s="515"/>
-      <c r="E6" s="515"/>
-      <c r="F6" s="515"/>
-      <c r="G6" s="515"/>
-      <c r="H6" s="515"/>
-      <c r="I6" s="515"/>
-      <c r="J6" s="515"/>
+      <c r="B6" s="523"/>
+      <c r="C6" s="523"/>
+      <c r="D6" s="523"/>
+      <c r="E6" s="523"/>
+      <c r="F6" s="523"/>
+      <c r="G6" s="523"/>
+      <c r="H6" s="523"/>
+      <c r="I6" s="523"/>
+      <c r="J6" s="523"/>
       <c r="K6" s="73"/>
       <c r="L6" s="73"/>
     </row>
     <row r="7" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="516">
+      <c r="A7" s="524">
         <v>0</v>
       </c>
-      <c r="B7" s="516"/>
-      <c r="C7" s="516"/>
-      <c r="D7" s="516"/>
-      <c r="E7" s="516"/>
-      <c r="F7" s="516"/>
-      <c r="G7" s="516"/>
-      <c r="H7" s="516"/>
-      <c r="I7" s="516"/>
-      <c r="J7" s="516"/>
+      <c r="B7" s="524"/>
+      <c r="C7" s="524"/>
+      <c r="D7" s="524"/>
+      <c r="E7" s="524"/>
+      <c r="F7" s="524"/>
+      <c r="G7" s="524"/>
+      <c r="H7" s="524"/>
+      <c r="I7" s="524"/>
+      <c r="J7" s="524"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="74"/>
@@ -7275,14 +7147,14 @@
       <c r="B9" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="C9" s="520">
+      <c r="C9" s="528">
         <f>+FORMATO!N2</f>
         <v>0</v>
       </c>
-      <c r="D9" s="520"/>
-      <c r="E9" s="520"/>
-      <c r="F9" s="520"/>
-      <c r="G9" s="520"/>
+      <c r="D9" s="528"/>
+      <c r="E9" s="528"/>
+      <c r="F9" s="528"/>
+      <c r="G9" s="528"/>
       <c r="H9" s="94" t="s">
         <v>19</v>
       </c>
@@ -7303,14 +7175,14 @@
       <c r="B10" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="C10" s="520">
+      <c r="C10" s="528">
         <f>+FORMATO!N3</f>
         <v>0</v>
       </c>
-      <c r="D10" s="520"/>
-      <c r="E10" s="520"/>
-      <c r="F10" s="520"/>
-      <c r="G10" s="520"/>
+      <c r="D10" s="528"/>
+      <c r="E10" s="528"/>
+      <c r="F10" s="528"/>
+      <c r="G10" s="528"/>
       <c r="H10" s="279" t="s">
         <v>132</v>
       </c>
@@ -7334,14 +7206,14 @@
       <c r="B11" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="C11" s="520">
+      <c r="C11" s="528">
         <f>+FORMATO!N4</f>
         <v>0</v>
       </c>
-      <c r="D11" s="520"/>
-      <c r="E11" s="520"/>
-      <c r="F11" s="520"/>
-      <c r="G11" s="520"/>
+      <c r="D11" s="528"/>
+      <c r="E11" s="528"/>
+      <c r="F11" s="528"/>
+      <c r="G11" s="528"/>
       <c r="H11" s="71" t="s">
         <v>16</v>
       </c>
@@ -7355,8 +7227,8 @@
       <c r="K11" s="15"/>
       <c r="L11" s="15"/>
       <c r="M11" s="15"/>
-      <c r="O11" s="521"/>
-      <c r="P11" s="521"/>
+      <c r="O11" s="513"/>
+      <c r="P11" s="513"/>
     </row>
     <row r="12" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="65" t="s">
@@ -7365,14 +7237,14 @@
       <c r="B12" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="C12" s="520">
+      <c r="C12" s="528">
         <f>+FORMATO!N5</f>
         <v>0</v>
       </c>
-      <c r="D12" s="520"/>
-      <c r="E12" s="520"/>
-      <c r="F12" s="520"/>
-      <c r="G12" s="520"/>
+      <c r="D12" s="528"/>
+      <c r="E12" s="528"/>
+      <c r="F12" s="528"/>
+      <c r="G12" s="528"/>
       <c r="H12" s="71" t="s">
         <v>21</v>
       </c>
@@ -7409,34 +7281,34 @@
       <c r="P13" s="16"/>
     </row>
     <row r="14" spans="1:16" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="522" t="s">
+      <c r="A14" s="514" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="523"/>
-      <c r="C14" s="523"/>
-      <c r="D14" s="523"/>
-      <c r="E14" s="523"/>
-      <c r="F14" s="523"/>
-      <c r="G14" s="523"/>
-      <c r="H14" s="523"/>
-      <c r="I14" s="523"/>
-      <c r="J14" s="524"/>
+      <c r="B14" s="515"/>
+      <c r="C14" s="515"/>
+      <c r="D14" s="515"/>
+      <c r="E14" s="515"/>
+      <c r="F14" s="515"/>
+      <c r="G14" s="515"/>
+      <c r="H14" s="515"/>
+      <c r="I14" s="515"/>
+      <c r="J14" s="516"/>
       <c r="K14" s="15"/>
       <c r="L14" s="15"/>
     </row>
     <row r="15" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="517" t="s">
+      <c r="A15" s="525" t="s">
         <v>151</v>
       </c>
-      <c r="B15" s="518"/>
-      <c r="C15" s="518"/>
-      <c r="D15" s="518"/>
-      <c r="E15" s="518"/>
-      <c r="F15" s="518"/>
-      <c r="G15" s="518"/>
-      <c r="H15" s="518"/>
-      <c r="I15" s="518"/>
-      <c r="J15" s="519"/>
+      <c r="B15" s="526"/>
+      <c r="C15" s="526"/>
+      <c r="D15" s="526"/>
+      <c r="E15" s="526"/>
+      <c r="F15" s="526"/>
+      <c r="G15" s="526"/>
+      <c r="H15" s="526"/>
+      <c r="I15" s="526"/>
+      <c r="J15" s="527"/>
       <c r="K15" s="15"/>
       <c r="L15" s="15"/>
     </row>
@@ -7478,7 +7350,7 @@
       <c r="D18" s="289" t="s">
         <v>0</v>
       </c>
-      <c r="E18" s="464">
+      <c r="E18" s="462">
         <f>+FORMATO!N15</f>
         <v>0</v>
       </c>
@@ -7506,7 +7378,7 @@
       <c r="D19" s="289" t="s">
         <v>0</v>
       </c>
-      <c r="E19" s="464">
+      <c r="E19" s="462">
         <f>+FORMATO!N16</f>
         <v>0</v>
       </c>
@@ -7537,7 +7409,7 @@
       <c r="D20" s="289" t="s">
         <v>0</v>
       </c>
-      <c r="E20" s="464">
+      <c r="E20" s="462">
         <f>+FORMATO!N17</f>
         <v>0</v>
       </c>
@@ -7612,10 +7484,10 @@
       <c r="B23" s="65"/>
       <c r="C23" s="65"/>
       <c r="D23" s="65"/>
-      <c r="E23" s="526" t="s">
+      <c r="E23" s="518" t="s">
         <v>51</v>
       </c>
-      <c r="F23" s="527"/>
+      <c r="F23" s="519"/>
       <c r="G23" s="105" t="s">
         <v>38</v>
       </c>
@@ -7641,10 +7513,10 @@
       <c r="B24" s="56"/>
       <c r="C24" s="108"/>
       <c r="D24" s="108"/>
-      <c r="E24" s="525" t="s">
+      <c r="E24" s="517" t="s">
         <v>144</v>
       </c>
-      <c r="F24" s="525"/>
+      <c r="F24" s="517"/>
       <c r="G24" s="109" t="s">
         <v>39</v>
       </c>
@@ -7672,10 +7544,10 @@
       <c r="B25" s="56"/>
       <c r="C25" s="108"/>
       <c r="D25" s="108"/>
-      <c r="E25" s="525" t="s">
+      <c r="E25" s="517" t="s">
         <v>143</v>
       </c>
-      <c r="F25" s="525"/>
+      <c r="F25" s="517"/>
       <c r="G25" s="109" t="s">
         <v>39</v>
       </c>
@@ -7702,10 +7574,10 @@
       <c r="B26" s="56"/>
       <c r="C26" s="108"/>
       <c r="D26" s="108"/>
-      <c r="E26" s="528" t="s">
+      <c r="E26" s="521" t="s">
         <v>70</v>
       </c>
-      <c r="F26" s="528"/>
+      <c r="F26" s="521"/>
       <c r="G26" s="112" t="s">
         <v>40</v>
       </c>
@@ -7903,18 +7775,18 @@
       <c r="X33" s="42"/>
     </row>
     <row r="34" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="529" t="s">
+      <c r="A34" s="522" t="s">
         <v>169</v>
       </c>
-      <c r="B34" s="529"/>
-      <c r="C34" s="529"/>
-      <c r="D34" s="529"/>
-      <c r="E34" s="529"/>
-      <c r="F34" s="529"/>
-      <c r="G34" s="529"/>
-      <c r="H34" s="529"/>
-      <c r="I34" s="529"/>
-      <c r="J34" s="529"/>
+      <c r="B34" s="522"/>
+      <c r="C34" s="522"/>
+      <c r="D34" s="522"/>
+      <c r="E34" s="522"/>
+      <c r="F34" s="522"/>
+      <c r="G34" s="522"/>
+      <c r="H34" s="522"/>
+      <c r="I34" s="522"/>
+      <c r="J34" s="522"/>
       <c r="K34" s="262"/>
       <c r="L34" s="262"/>
       <c r="M34" s="23"/>
@@ -7929,18 +7801,18 @@
       <c r="X34" s="42"/>
     </row>
     <row r="35" spans="1:24" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="514" t="s">
+      <c r="A35" s="520" t="s">
         <v>170</v>
       </c>
-      <c r="B35" s="514"/>
-      <c r="C35" s="514"/>
-      <c r="D35" s="514"/>
-      <c r="E35" s="514"/>
-      <c r="F35" s="514"/>
-      <c r="G35" s="514"/>
-      <c r="H35" s="514"/>
-      <c r="I35" s="514"/>
-      <c r="J35" s="514"/>
+      <c r="B35" s="520"/>
+      <c r="C35" s="520"/>
+      <c r="D35" s="520"/>
+      <c r="E35" s="520"/>
+      <c r="F35" s="520"/>
+      <c r="G35" s="520"/>
+      <c r="H35" s="520"/>
+      <c r="I35" s="520"/>
+      <c r="J35" s="520"/>
       <c r="M35" s="23"/>
       <c r="N35" s="29"/>
       <c r="P35" s="39"/>
@@ -7953,18 +7825,18 @@
       <c r="X35" s="42"/>
     </row>
     <row r="36" spans="1:24" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="514" t="s">
+      <c r="A36" s="520" t="s">
         <v>171</v>
       </c>
-      <c r="B36" s="514"/>
-      <c r="C36" s="514"/>
-      <c r="D36" s="514"/>
-      <c r="E36" s="514"/>
-      <c r="F36" s="514"/>
-      <c r="G36" s="514"/>
-      <c r="H36" s="514"/>
-      <c r="I36" s="514"/>
-      <c r="J36" s="514"/>
+      <c r="B36" s="520"/>
+      <c r="C36" s="520"/>
+      <c r="D36" s="520"/>
+      <c r="E36" s="520"/>
+      <c r="F36" s="520"/>
+      <c r="G36" s="520"/>
+      <c r="H36" s="520"/>
+      <c r="I36" s="520"/>
+      <c r="J36" s="520"/>
       <c r="K36" s="263"/>
       <c r="L36" s="263"/>
       <c r="M36" s="48"/>
@@ -7979,18 +7851,18 @@
       <c r="X36" s="42"/>
     </row>
     <row r="37" spans="1:24" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="514" t="s">
+      <c r="A37" s="520" t="s">
         <v>172</v>
       </c>
-      <c r="B37" s="514"/>
-      <c r="C37" s="514"/>
-      <c r="D37" s="514"/>
-      <c r="E37" s="514"/>
-      <c r="F37" s="514"/>
-      <c r="G37" s="514"/>
-      <c r="H37" s="514"/>
-      <c r="I37" s="514"/>
-      <c r="J37" s="514"/>
+      <c r="B37" s="520"/>
+      <c r="C37" s="520"/>
+      <c r="D37" s="520"/>
+      <c r="E37" s="520"/>
+      <c r="F37" s="520"/>
+      <c r="G37" s="520"/>
+      <c r="H37" s="520"/>
+      <c r="I37" s="520"/>
+      <c r="J37" s="520"/>
       <c r="N37" s="29"/>
       <c r="P37" s="39"/>
       <c r="Q37" s="28"/>
@@ -8002,18 +7874,18 @@
       <c r="X37" s="31"/>
     </row>
     <row r="38" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="514" t="s">
+      <c r="A38" s="520" t="s">
         <v>173</v>
       </c>
-      <c r="B38" s="514"/>
-      <c r="C38" s="514"/>
-      <c r="D38" s="514"/>
-      <c r="E38" s="514"/>
-      <c r="F38" s="514"/>
-      <c r="G38" s="514"/>
-      <c r="H38" s="514"/>
-      <c r="I38" s="514"/>
-      <c r="J38" s="514"/>
+      <c r="B38" s="520"/>
+      <c r="C38" s="520"/>
+      <c r="D38" s="520"/>
+      <c r="E38" s="520"/>
+      <c r="F38" s="520"/>
+      <c r="G38" s="520"/>
+      <c r="H38" s="520"/>
+      <c r="I38" s="520"/>
+      <c r="J38" s="520"/>
       <c r="K38" s="263"/>
       <c r="L38" s="263"/>
       <c r="M38" s="263"/>
@@ -8331,15 +8203,6 @@
     <protectedRange sqref="E9 D11:D12 D10:E10" name="Rango3_3_1_1_1_1_1_2_1_1"/>
   </protectedRanges>
   <mergeCells count="19">
-    <mergeCell ref="O11:P11"/>
-    <mergeCell ref="A14:J14"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="A36:J36"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="A34:J34"/>
-    <mergeCell ref="A35:J35"/>
     <mergeCell ref="A38:J38"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A7:J7"/>
@@ -8350,6 +8213,15 @@
     <mergeCell ref="C10:G10"/>
     <mergeCell ref="C11:G11"/>
     <mergeCell ref="C12:G12"/>
+    <mergeCell ref="O11:P11"/>
+    <mergeCell ref="A14:J14"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="A36:J36"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="A34:J34"/>
+    <mergeCell ref="A35:J35"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
@@ -8389,20 +8261,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="538" t="s">
+      <c r="A1" s="529" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="538"/>
-      <c r="C1" s="538"/>
-      <c r="D1" s="538"/>
-      <c r="E1" s="538"/>
-      <c r="F1" s="538"/>
-      <c r="G1" s="538"/>
-      <c r="H1" s="538"/>
-      <c r="I1" s="538"/>
-      <c r="J1" s="538"/>
-      <c r="K1" s="538"/>
-      <c r="L1" s="538"/>
+      <c r="B1" s="529"/>
+      <c r="C1" s="529"/>
+      <c r="D1" s="529"/>
+      <c r="E1" s="529"/>
+      <c r="F1" s="529"/>
+      <c r="G1" s="529"/>
+      <c r="H1" s="529"/>
+      <c r="I1" s="529"/>
+      <c r="J1" s="529"/>
+      <c r="K1" s="529"/>
+      <c r="L1" s="529"/>
       <c r="T1" s="295" t="s">
         <v>61</v>
       </c>
@@ -8532,10 +8404,10 @@
     </row>
     <row r="8" spans="1:20" ht="25.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="60"/>
-      <c r="B8" s="531" t="s">
+      <c r="B8" s="545" t="s">
         <v>51</v>
       </c>
-      <c r="C8" s="532"/>
+      <c r="C8" s="546"/>
       <c r="D8" s="284" t="s">
         <v>38</v>
       </c>
@@ -8561,10 +8433,10 @@
     </row>
     <row r="9" spans="1:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="60"/>
-      <c r="B9" s="478" t="s">
+      <c r="B9" s="480" t="s">
         <v>52</v>
       </c>
-      <c r="C9" s="479"/>
+      <c r="C9" s="481"/>
       <c r="D9" s="61" t="s">
         <v>39</v>
       </c>
@@ -8591,10 +8463,10 @@
     </row>
     <row r="10" spans="1:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="60"/>
-      <c r="B10" s="478" t="s">
+      <c r="B10" s="480" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="479"/>
+      <c r="C10" s="481"/>
       <c r="D10" s="61" t="s">
         <v>39</v>
       </c>
@@ -8622,10 +8494,10 @@
     </row>
     <row r="11" spans="1:20" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="60"/>
-      <c r="B11" s="533" t="s">
+      <c r="B11" s="547" t="s">
         <v>54</v>
       </c>
-      <c r="C11" s="533"/>
+      <c r="C11" s="547"/>
       <c r="D11" s="61" t="s">
         <v>39</v>
       </c>
@@ -8710,34 +8582,34 @@
     </row>
     <row r="14" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="107"/>
-      <c r="B14" s="546" t="s">
+      <c r="B14" s="537" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="547"/>
-      <c r="D14" s="548"/>
-      <c r="E14" s="541" t="s">
+      <c r="C14" s="538"/>
+      <c r="D14" s="539"/>
+      <c r="E14" s="532" t="s">
         <v>135</v>
       </c>
-      <c r="F14" s="541" t="s">
+      <c r="F14" s="532" t="s">
         <v>136</v>
       </c>
-      <c r="G14" s="543" t="s">
+      <c r="G14" s="534" t="s">
         <v>137</v>
       </c>
       <c r="H14" s="290"/>
-      <c r="I14" s="545" t="s">
+      <c r="I14" s="536" t="s">
         <v>142</v>
       </c>
-      <c r="J14" s="545"/>
+      <c r="J14" s="536"/>
       <c r="L14" s="339"/>
       <c r="M14" s="21"/>
       <c r="N14" s="23"/>
       <c r="O14" s="27"/>
       <c r="P14" s="27"/>
       <c r="Q14" s="26"/>
-      <c r="R14" s="539"/>
-      <c r="S14" s="539"/>
-      <c r="T14" s="539"/>
+      <c r="R14" s="530"/>
+      <c r="S14" s="530"/>
+      <c r="T14" s="530"/>
     </row>
     <row r="15" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="107"/>
@@ -8748,9 +8620,9 @@
         <v>28</v>
       </c>
       <c r="D15" s="62"/>
-      <c r="E15" s="542"/>
-      <c r="F15" s="542"/>
-      <c r="G15" s="544"/>
+      <c r="E15" s="533"/>
+      <c r="F15" s="533"/>
+      <c r="G15" s="535"/>
       <c r="H15" s="341"/>
       <c r="I15" s="140" t="s">
         <v>138</v>
@@ -8909,15 +8781,15 @@
       <c r="L19" s="346"/>
       <c r="M19" s="298"/>
       <c r="N19" s="23"/>
-      <c r="O19" s="540"/>
-      <c r="P19" s="540"/>
-      <c r="Q19" s="540"/>
-      <c r="R19" s="540"/>
-      <c r="S19" s="540"/>
+      <c r="O19" s="531"/>
+      <c r="P19" s="531"/>
+      <c r="Q19" s="531"/>
+      <c r="R19" s="531"/>
+      <c r="S19" s="531"/>
       <c r="T19" s="35"/>
-      <c r="U19" s="534"/>
-      <c r="V19" s="534"/>
-      <c r="W19" s="534"/>
+      <c r="U19" s="540"/>
+      <c r="V19" s="540"/>
+      <c r="W19" s="540"/>
     </row>
     <row r="20" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="107"/>
@@ -8956,16 +8828,16 @@
       <c r="R20" s="35"/>
       <c r="S20" s="35"/>
       <c r="T20" s="35"/>
-      <c r="U20" s="534"/>
-      <c r="V20" s="534"/>
-      <c r="W20" s="534"/>
+      <c r="U20" s="540"/>
+      <c r="V20" s="540"/>
+      <c r="W20" s="540"/>
     </row>
     <row r="21" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="107"/>
-      <c r="B21" s="536" t="s">
+      <c r="B21" s="542" t="s">
         <v>66</v>
       </c>
-      <c r="C21" s="537"/>
+      <c r="C21" s="543"/>
       <c r="D21" s="62"/>
       <c r="E21" s="301">
         <f>SUM(E16:E20)</f>
@@ -9029,10 +8901,10 @@
       <c r="A23" s="260" t="s">
         <v>77</v>
       </c>
-      <c r="B23" s="531" t="s">
+      <c r="B23" s="545" t="s">
         <v>51</v>
       </c>
-      <c r="C23" s="532"/>
+      <c r="C23" s="546"/>
       <c r="D23" s="284" t="s">
         <v>38</v>
       </c>
@@ -9059,10 +8931,10 @@
       <c r="A24" s="261" t="s">
         <v>129</v>
       </c>
-      <c r="B24" s="478" t="s">
+      <c r="B24" s="480" t="s">
         <v>144</v>
       </c>
-      <c r="C24" s="479"/>
+      <c r="C24" s="481"/>
       <c r="D24" s="61" t="s">
         <v>39</v>
       </c>
@@ -9088,10 +8960,10 @@
       <c r="A25" s="261" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="473" t="s">
+      <c r="B25" s="504" t="s">
         <v>146</v>
       </c>
-      <c r="C25" s="474"/>
+      <c r="C25" s="505"/>
       <c r="D25" s="64" t="s">
         <v>39</v>
       </c>
@@ -9117,10 +8989,10 @@
       <c r="A26" s="61" t="s">
         <v>63</v>
       </c>
-      <c r="B26" s="473" t="s">
+      <c r="B26" s="504" t="s">
         <v>147</v>
       </c>
-      <c r="C26" s="474"/>
+      <c r="C26" s="505"/>
       <c r="D26" s="64" t="s">
         <v>39</v>
       </c>
@@ -9152,10 +9024,10 @@
       <c r="A27" s="61" t="s">
         <v>64</v>
       </c>
-      <c r="B27" s="473" t="s">
+      <c r="B27" s="504" t="s">
         <v>148</v>
       </c>
-      <c r="C27" s="474"/>
+      <c r="C27" s="505"/>
       <c r="D27" s="64" t="s">
         <v>39</v>
       </c>
@@ -9184,10 +9056,10 @@
       <c r="A28" s="61" t="s">
         <v>65</v>
       </c>
-      <c r="B28" s="473" t="s">
+      <c r="B28" s="504" t="s">
         <v>149</v>
       </c>
-      <c r="C28" s="474"/>
+      <c r="C28" s="505"/>
       <c r="D28" s="64" t="s">
         <v>39</v>
       </c>
@@ -9216,10 +9088,10 @@
       <c r="A29" s="61" t="s">
         <v>130</v>
       </c>
-      <c r="B29" s="473" t="s">
+      <c r="B29" s="504" t="s">
         <v>141</v>
       </c>
-      <c r="C29" s="474"/>
+      <c r="C29" s="505"/>
       <c r="D29" s="64" t="s">
         <v>40</v>
       </c>
@@ -9246,10 +9118,10 @@
     </row>
     <row r="30" spans="1:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="61"/>
-      <c r="B30" s="473" t="s">
+      <c r="B30" s="504" t="s">
         <v>145</v>
       </c>
-      <c r="C30" s="477"/>
+      <c r="C30" s="506"/>
       <c r="D30" s="64" t="s">
         <v>40</v>
       </c>
@@ -9399,8 +9271,8 @@
     </row>
     <row r="37" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="44"/>
-      <c r="B37" s="535"/>
-      <c r="C37" s="535"/>
+      <c r="B37" s="541"/>
+      <c r="C37" s="541"/>
       <c r="J37" s="42"/>
       <c r="M37" s="15"/>
       <c r="N37" s="23"/>
@@ -9467,17 +9339,17 @@
       <c r="W41" s="42"/>
     </row>
     <row r="42" spans="1:23" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="530"/>
-      <c r="B42" s="530"/>
-      <c r="C42" s="530"/>
-      <c r="D42" s="530"/>
-      <c r="E42" s="530"/>
-      <c r="F42" s="530"/>
-      <c r="G42" s="530"/>
-      <c r="H42" s="530"/>
-      <c r="I42" s="530"/>
-      <c r="J42" s="530"/>
-      <c r="K42" s="530"/>
+      <c r="A42" s="544"/>
+      <c r="B42" s="544"/>
+      <c r="C42" s="544"/>
+      <c r="D42" s="544"/>
+      <c r="E42" s="544"/>
+      <c r="F42" s="544"/>
+      <c r="G42" s="544"/>
+      <c r="H42" s="544"/>
+      <c r="I42" s="544"/>
+      <c r="J42" s="544"/>
+      <c r="K42" s="544"/>
       <c r="L42" s="42"/>
       <c r="M42" s="15"/>
       <c r="N42" s="48"/>
@@ -9599,6 +9471,21 @@
     <protectedRange sqref="C2" name="Rango3_3_1_1_1_1_1_1_1_1_1_1"/>
   </protectedRanges>
   <mergeCells count="25">
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="U19:W20"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="R14:T14"/>
@@ -9609,21 +9496,6 @@
     <mergeCell ref="G14:G15"/>
     <mergeCell ref="I14:J14"/>
     <mergeCell ref="B14:D14"/>
-    <mergeCell ref="U19:W20"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="A42:K42"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
   </mergeCells>
   <conditionalFormatting sqref="F30:F31">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
@@ -9696,16 +9568,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="557"/>
-      <c r="B1" s="558"/>
-      <c r="C1" s="563" t="s">
+      <c r="A1" s="548"/>
+      <c r="B1" s="549"/>
+      <c r="C1" s="554" t="s">
         <v>83</v>
       </c>
-      <c r="D1" s="564"/>
-      <c r="E1" s="564"/>
-      <c r="F1" s="564"/>
-      <c r="G1" s="564"/>
-      <c r="H1" s="565"/>
+      <c r="D1" s="555"/>
+      <c r="E1" s="555"/>
+      <c r="F1" s="555"/>
+      <c r="G1" s="555"/>
+      <c r="H1" s="556"/>
       <c r="I1" s="167" t="s">
         <v>84</v>
       </c>
@@ -9714,14 +9586,14 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="559"/>
-      <c r="B2" s="560"/>
-      <c r="C2" s="566"/>
-      <c r="D2" s="567"/>
-      <c r="E2" s="567"/>
-      <c r="F2" s="567"/>
-      <c r="G2" s="567"/>
-      <c r="H2" s="568"/>
+      <c r="A2" s="550"/>
+      <c r="B2" s="551"/>
+      <c r="C2" s="557"/>
+      <c r="D2" s="558"/>
+      <c r="E2" s="558"/>
+      <c r="F2" s="558"/>
+      <c r="G2" s="558"/>
+      <c r="H2" s="559"/>
       <c r="I2" s="167" t="s">
         <v>86</v>
       </c>
@@ -9730,14 +9602,14 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="559"/>
-      <c r="B3" s="560"/>
-      <c r="C3" s="566"/>
-      <c r="D3" s="567"/>
-      <c r="E3" s="567"/>
-      <c r="F3" s="567"/>
-      <c r="G3" s="567"/>
-      <c r="H3" s="568"/>
+      <c r="A3" s="550"/>
+      <c r="B3" s="551"/>
+      <c r="C3" s="557"/>
+      <c r="D3" s="558"/>
+      <c r="E3" s="558"/>
+      <c r="F3" s="558"/>
+      <c r="G3" s="558"/>
+      <c r="H3" s="559"/>
       <c r="I3" s="167" t="s">
         <v>87</v>
       </c>
@@ -9746,14 +9618,14 @@
       </c>
     </row>
     <row r="4" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="561"/>
-      <c r="B4" s="562"/>
-      <c r="C4" s="569"/>
-      <c r="D4" s="570"/>
-      <c r="E4" s="570"/>
-      <c r="F4" s="570"/>
-      <c r="G4" s="570"/>
-      <c r="H4" s="571"/>
+      <c r="A4" s="552"/>
+      <c r="B4" s="553"/>
+      <c r="C4" s="560"/>
+      <c r="D4" s="561"/>
+      <c r="E4" s="561"/>
+      <c r="F4" s="561"/>
+      <c r="G4" s="561"/>
+      <c r="H4" s="562"/>
       <c r="I4" s="167" t="s">
         <v>88</v>
       </c>
@@ -9766,17 +9638,17 @@
       <c r="A6" s="169" t="s">
         <v>90</v>
       </c>
-      <c r="B6" s="573" t="s">
+      <c r="B6" s="564" t="s">
         <v>122</v>
       </c>
-      <c r="C6" s="574"/>
-      <c r="D6" s="574"/>
-      <c r="E6" s="574"/>
-      <c r="F6" s="574"/>
-      <c r="G6" s="574"/>
-      <c r="H6" s="574"/>
-      <c r="I6" s="574"/>
-      <c r="J6" s="575"/>
+      <c r="C6" s="565"/>
+      <c r="D6" s="565"/>
+      <c r="E6" s="565"/>
+      <c r="F6" s="565"/>
+      <c r="G6" s="565"/>
+      <c r="H6" s="565"/>
+      <c r="I6" s="565"/>
+      <c r="J6" s="566"/>
     </row>
     <row r="7" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="169" t="s">
@@ -10573,12 +10445,12 @@
       <c r="M42" s="143"/>
     </row>
     <row r="43" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A43" s="576" t="s">
+      <c r="A43" s="567" t="s">
         <v>162</v>
       </c>
-      <c r="B43" s="576"/>
-      <c r="C43" s="576"/>
-      <c r="D43" s="576"/>
+      <c r="B43" s="567"/>
+      <c r="C43" s="567"/>
+      <c r="D43" s="567"/>
       <c r="E43" s="177"/>
       <c r="F43" s="177"/>
       <c r="G43" s="177"/>
@@ -10588,10 +10460,10 @@
       <c r="M43" s="143"/>
     </row>
     <row r="44" spans="1:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="572" t="s">
+      <c r="A44" s="563" t="s">
         <v>115</v>
       </c>
-      <c r="B44" s="572"/>
+      <c r="B44" s="563"/>
       <c r="C44" s="183" t="s">
         <v>116</v>
       </c>
@@ -10688,19 +10560,19 @@
       <c r="A51" s="379" t="s">
         <v>153</v>
       </c>
-      <c r="B51" s="549" t="s">
+      <c r="B51" s="568" t="s">
         <v>154</v>
       </c>
-      <c r="C51" s="550"/>
+      <c r="C51" s="569"/>
       <c r="D51" s="380"/>
-      <c r="E51" s="551" t="s">
+      <c r="E51" s="570" t="s">
         <v>155</v>
       </c>
-      <c r="F51" s="551"/>
-      <c r="G51" s="552" t="s">
+      <c r="F51" s="570"/>
+      <c r="G51" s="571" t="s">
         <v>156</v>
       </c>
-      <c r="H51" s="553"/>
+      <c r="H51" s="572"/>
       <c r="I51" s="171"/>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -10718,19 +10590,19 @@
       <c r="A53" s="381" t="s">
         <v>157</v>
       </c>
-      <c r="B53" s="554">
+      <c r="B53" s="573">
         <v>45604</v>
       </c>
-      <c r="C53" s="555"/>
+      <c r="C53" s="574"/>
       <c r="D53" s="171"/>
-      <c r="E53" s="556" t="s">
+      <c r="E53" s="575" t="s">
         <v>158</v>
       </c>
-      <c r="F53" s="556"/>
-      <c r="G53" s="554">
+      <c r="F53" s="575"/>
+      <c r="G53" s="573">
         <v>45605</v>
       </c>
-      <c r="H53" s="555"/>
+      <c r="H53" s="574"/>
       <c r="I53" s="171"/>
     </row>
     <row r="54" spans="1:9" ht="13.8" x14ac:dyDescent="0.3">
@@ -10739,17 +10611,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="WnakG9b2+KFY7KUJ1FRTPtBZcRMVBGtSwjnmFUbl3JunMT2lACh16v6BaQQSu6NvxTQ8y3ZAFE75ggf6peBN9A==" saltValue="1kkdm0zTKwaCrCcKsSMpLQ==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="11">
-    <mergeCell ref="A1:B4"/>
-    <mergeCell ref="C1:H4"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="B6:J6"/>
-    <mergeCell ref="A43:D43"/>
     <mergeCell ref="B51:C51"/>
     <mergeCell ref="E51:F51"/>
     <mergeCell ref="G51:H51"/>
     <mergeCell ref="B53:C53"/>
     <mergeCell ref="E53:F53"/>
     <mergeCell ref="G53:H53"/>
+    <mergeCell ref="A1:B4"/>
+    <mergeCell ref="C1:H4"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="B6:J6"/>
+    <mergeCell ref="A43:D43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10780,14 +10652,14 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="141"/>
-      <c r="B2" s="577" t="s">
+      <c r="B2" s="576" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="577"/>
-      <c r="D2" s="577"/>
-      <c r="E2" s="577"/>
-      <c r="F2" s="577"/>
-      <c r="G2" s="577"/>
+      <c r="C2" s="576"/>
+      <c r="D2" s="576"/>
+      <c r="E2" s="576"/>
+      <c r="F2" s="576"/>
+      <c r="G2" s="576"/>
       <c r="H2" s="141"/>
       <c r="I2" s="141"/>
       <c r="J2" s="141"/>
@@ -10841,8 +10713,8 @@
       <c r="F6" s="141"/>
       <c r="G6" s="141"/>
       <c r="H6" s="141"/>
-      <c r="I6" s="578"/>
-      <c r="J6" s="579"/>
+      <c r="I6" s="577"/>
+      <c r="J6" s="578"/>
       <c r="K6" s="141"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -11160,10 +11032,10 @@
     </row>
     <row r="24" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="141"/>
-      <c r="B24" s="478" t="s">
+      <c r="B24" s="480" t="s">
         <v>68</v>
       </c>
-      <c r="C24" s="479"/>
+      <c r="C24" s="481"/>
       <c r="D24" s="191">
         <f>+DATOS!F24</f>
         <v>0</v>
@@ -11174,10 +11046,10 @@
       </c>
     </row>
     <row r="25" spans="1:11" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="580" t="s">
+      <c r="B25" s="579" t="s">
         <v>71</v>
       </c>
-      <c r="C25" s="581"/>
+      <c r="C25" s="580"/>
       <c r="D25" s="192">
         <f>+DATOS!G26</f>
         <v>0</v>
@@ -11263,21 +11135,21 @@
       <c r="A7" s="166" t="s">
         <v>165</v>
       </c>
-      <c r="B7" s="582">
+      <c r="B7" s="581">
         <v>9.0531621221234589E-3</v>
       </c>
-      <c r="C7" s="582"/>
-      <c r="D7" s="582"/>
+      <c r="C7" s="581"/>
+      <c r="D7" s="581"/>
     </row>
     <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="166" t="s">
         <v>166</v>
       </c>
-      <c r="B8" s="583">
+      <c r="B8" s="582">
         <v>1.7951817913661365E-3</v>
       </c>
-      <c r="C8" s="583"/>
-      <c r="D8" s="583"/>
+      <c r="C8" s="582"/>
+      <c r="D8" s="582"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="kx95A5hTynsyU7blcEsS5tlD7yCb2kjCkGJLwcTBpdgNp98Z2L+KdYTx6mJJYTWOzhHnJD0gTotl9NQF8d13pA==" saltValue="fYngoKT1w/kUCRXt4zKmow==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
@@ -11305,10 +11177,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="584" t="s">
+      <c r="A2" s="583" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="584"/>
+      <c r="B2" s="583"/>
       <c r="C2" s="5" t="s">
         <v>11</v>
       </c>

</xml_diff>